<commit_message>
filtered transaction history to include only shadow ones
</commit_message>
<xml_diff>
--- a/AAII.xlsx
+++ b/AAII.xlsx
@@ -9,14 +9,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="KGDmQxXIW+PcKGbAZTcrk/pIEenyBBf3kY9/OhaqUFw="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="zbRaNs827EUg825F1vh205JS9/tT4fA77JY+qRLrasY="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="98">
   <si>
     <t>Company</t>
   </si>
@@ -99,7 +99,7 @@
     <t>CVLG</t>
   </si>
   <si>
-    <t>(4/23/26) Covenant Logistics Group, Inc. (CVLG)</t>
+    <t>News Archive for CVLG</t>
   </si>
   <si>
     <t>DMC Global Inc.</t>
@@ -114,7 +114,7 @@
     <t>Earnings probation 2025q4</t>
   </si>
   <si>
-    <t>News Archive for BOOM</t>
+    <t>(4/30/26) DMC Global Inc. (BOOM)</t>
   </si>
   <si>
     <t>Ennis, Inc.</t>
@@ -123,7 +123,7 @@
     <t>EBF</t>
   </si>
   <si>
-    <t>(4/20/26) Ennis, Inc. (EBF)</t>
+    <t>News Archive for EBF</t>
   </si>
   <si>
     <t>Escalade, Incorporated</t>
@@ -132,7 +132,7 @@
     <t>ESCA</t>
   </si>
   <si>
-    <t>News Archive for ESCA</t>
+    <t>(4/30/26) Escalade, Incorporated (ESCA)</t>
   </si>
   <si>
     <t>Euroseas Ltd.</t>
@@ -192,7 +192,7 @@
     <t>Earnings probation 2025Q3</t>
   </si>
   <si>
-    <t>(4/20/26) Lakeland Industries, Inc. (LAKE)</t>
+    <t>News Archive for LAKE</t>
   </si>
   <si>
     <t>Mistras Group, Inc.</t>
@@ -231,7 +231,7 @@
     <t>NCSM</t>
   </si>
   <si>
-    <t>News Archive for NCSM</t>
+    <t>(4/29/26) NCS Multistage Holdings, Inc. (NCSM)</t>
   </si>
   <si>
     <t>Oil States International, Inc.</t>
@@ -276,7 +276,7 @@
     <t>RCKY</t>
   </si>
   <si>
-    <t>News Archive for RCKY</t>
+    <t>(4/28/26) Rocky Brands, Inc. (RCKY)</t>
   </si>
   <si>
     <t>Saga Communications, Inc.</t>
@@ -294,16 +294,7 @@
     <t>SDHC</t>
   </si>
   <si>
-    <t>News Archive for SDHC</t>
-  </si>
-  <si>
-    <t>StealthGas Inc.</t>
-  </si>
-  <si>
-    <t>GASS</t>
-  </si>
-  <si>
-    <t>News Archive for GASS</t>
+    <t>(4/29/26) Smith Douglas Homes Corp. (SDHC)</t>
   </si>
   <si>
     <t>The Eastern Company</t>
@@ -627,7 +618,7 @@
         <v>12</v>
       </c>
       <c r="C2" s="3">
-        <v>4.55</v>
+        <v>4.6</v>
       </c>
       <c r="D2" s="3">
         <v>5.64</v>
@@ -636,16 +627,16 @@
         <v>4.25</v>
       </c>
       <c r="F2" s="2">
-        <v>46.3</v>
+        <v>46.9</v>
       </c>
       <c r="G2" s="2">
-        <v>13.8</v>
+        <v>13.9</v>
       </c>
       <c r="H2" s="3">
-        <v>0.74</v>
+        <v>0.75</v>
       </c>
       <c r="I2" s="4">
-        <v>47.0</v>
+        <v>48.0</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>13</v>
@@ -662,25 +653,25 @@
         <v>16</v>
       </c>
       <c r="C3" s="3">
-        <v>5.84</v>
+        <v>6.23</v>
       </c>
       <c r="D3" s="3">
         <v>6.79</v>
       </c>
       <c r="E3" s="3">
-        <v>2.48</v>
+        <v>2.56</v>
       </c>
       <c r="F3" s="2">
-        <v>241.0</v>
+        <v>264.2</v>
       </c>
       <c r="G3" s="2">
-        <v>5.7</v>
+        <v>6.2</v>
       </c>
       <c r="H3" s="3">
-        <v>0.52</v>
+        <v>0.57</v>
       </c>
       <c r="I3" s="4">
-        <v>81.0</v>
+        <v>88.0</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>13</v>
@@ -697,7 +688,7 @@
         <v>19</v>
       </c>
       <c r="C4" s="3">
-        <v>1.93</v>
+        <v>2.09</v>
       </c>
       <c r="D4" s="3">
         <v>2.65</v>
@@ -706,16 +697,16 @@
         <v>1.66</v>
       </c>
       <c r="F4" s="2">
-        <v>18.6</v>
+        <v>19.9</v>
       </c>
       <c r="G4" s="2">
-        <v>5.4</v>
+        <v>5.7</v>
       </c>
       <c r="H4" s="3">
         <v>0.04</v>
       </c>
       <c r="I4" s="4">
-        <v>42.0</v>
+        <v>49.0</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>20</v>
@@ -732,7 +723,7 @@
         <v>23</v>
       </c>
       <c r="C5" s="3">
-        <v>28.1</v>
+        <v>26.61</v>
       </c>
       <c r="D5" s="3">
         <v>28.69</v>
@@ -741,16 +732,16 @@
         <v>14.48</v>
       </c>
       <c r="F5" s="2">
-        <v>249.1</v>
+        <v>238.9</v>
       </c>
       <c r="G5" s="2">
-        <v>21.8</v>
+        <v>20.9</v>
       </c>
       <c r="H5" s="3">
-        <v>1.51</v>
+        <v>1.45</v>
       </c>
       <c r="I5" s="4">
-        <v>87.0</v>
+        <v>88.0</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>24</v>
@@ -764,25 +755,25 @@
         <v>26</v>
       </c>
       <c r="C6" s="3">
-        <v>34.07</v>
+        <v>33.72</v>
       </c>
       <c r="D6" s="3">
-        <v>34.16</v>
+        <v>35.91</v>
       </c>
       <c r="E6" s="3">
         <v>18.0</v>
       </c>
       <c r="F6" s="2">
-        <v>854.9</v>
+        <v>874.7</v>
       </c>
       <c r="G6" s="2">
-        <v>212.9</v>
+        <v>217.9</v>
       </c>
       <c r="H6" s="3">
-        <v>2.11</v>
+        <v>2.16</v>
       </c>
       <c r="I6" s="4">
-        <v>90.0</v>
+        <v>94.0</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>27</v>
@@ -796,7 +787,7 @@
         <v>29</v>
       </c>
       <c r="C7" s="3">
-        <v>6.41</v>
+        <v>8.39</v>
       </c>
       <c r="D7" s="3">
         <v>9.2</v>
@@ -805,16 +796,16 @@
         <v>4.69</v>
       </c>
       <c r="F7" s="2">
-        <v>131.2</v>
+        <v>126.5</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>30</v>
       </c>
       <c r="H7" s="3">
-        <v>0.54</v>
+        <v>0.52</v>
       </c>
       <c r="I7" s="4">
-        <v>32.0</v>
+        <v>24.0</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>31</v>
@@ -831,7 +822,7 @@
         <v>34</v>
       </c>
       <c r="C8" s="3">
-        <v>20.33</v>
+        <v>21.09</v>
       </c>
       <c r="D8" s="3">
         <v>22.36</v>
@@ -840,16 +831,16 @@
         <v>16.3</v>
       </c>
       <c r="F8" s="2">
-        <v>514.2</v>
+        <v>528.1</v>
       </c>
       <c r="G8" s="2">
-        <v>12.3</v>
+        <v>12.6</v>
       </c>
       <c r="H8" s="3">
-        <v>1.68</v>
+        <v>1.73</v>
       </c>
       <c r="I8" s="4">
-        <v>70.0</v>
+        <v>76.0</v>
       </c>
       <c r="K8" s="2" t="s">
         <v>35</v>
@@ -863,7 +854,7 @@
         <v>37</v>
       </c>
       <c r="C9" s="3">
-        <v>18.09</v>
+        <v>18.19</v>
       </c>
       <c r="D9" s="3">
         <v>19.11</v>
@@ -872,16 +863,16 @@
         <v>11.41</v>
       </c>
       <c r="F9" s="2">
-        <v>247.8</v>
+        <v>256.1</v>
       </c>
       <c r="G9" s="2">
-        <v>18.3</v>
+        <v>18.9</v>
       </c>
       <c r="H9" s="3">
-        <v>1.43</v>
+        <v>1.48</v>
       </c>
       <c r="I9" s="4">
-        <v>87.0</v>
+        <v>92.0</v>
       </c>
       <c r="K9" s="2" t="s">
         <v>38</v>
@@ -895,22 +886,22 @@
         <v>40</v>
       </c>
       <c r="C10" s="3">
-        <v>68.03</v>
+        <v>69.96</v>
       </c>
       <c r="D10" s="3">
         <v>74.75</v>
       </c>
       <c r="E10" s="3">
-        <v>30.38</v>
+        <v>30.72</v>
       </c>
       <c r="F10" s="2">
-        <v>480.0</v>
+        <v>494.0</v>
       </c>
       <c r="G10" s="2">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
       <c r="H10" s="3">
-        <v>1.27</v>
+        <v>1.31</v>
       </c>
       <c r="I10" s="4">
         <v>74.0</v>
@@ -927,25 +918,25 @@
         <v>43</v>
       </c>
       <c r="C11" s="3">
-        <v>18.83</v>
+        <v>18.94</v>
       </c>
       <c r="D11" s="3">
-        <v>18.86</v>
+        <v>18.95</v>
       </c>
       <c r="E11" s="3">
-        <v>12.0</v>
+        <v>12.14</v>
       </c>
       <c r="F11" s="2">
-        <v>123.4</v>
+        <v>124.1</v>
       </c>
       <c r="G11" s="2">
-        <v>17.1</v>
+        <v>17.2</v>
       </c>
       <c r="H11" s="3">
         <v>0.7</v>
       </c>
       <c r="I11" s="4">
-        <v>72.0</v>
+        <v>74.0</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>13</v>
@@ -962,7 +953,7 @@
         <v>46</v>
       </c>
       <c r="C12" s="3">
-        <v>20.52</v>
+        <v>20.62</v>
       </c>
       <c r="D12" s="3">
         <v>24.37</v>
@@ -971,16 +962,16 @@
         <v>14.0</v>
       </c>
       <c r="F12" s="2">
-        <v>145.9</v>
+        <v>146.4</v>
       </c>
       <c r="G12" s="2">
-        <v>9.2</v>
+        <v>9.3</v>
       </c>
       <c r="H12" s="3">
         <v>1.03</v>
       </c>
       <c r="I12" s="4">
-        <v>52.0</v>
+        <v>47.0</v>
       </c>
       <c r="K12" s="2" t="s">
         <v>47</v>
@@ -994,7 +985,7 @@
         <v>49</v>
       </c>
       <c r="C13" s="3">
-        <v>17.42</v>
+        <v>18.47</v>
       </c>
       <c r="D13" s="3">
         <v>20.38</v>
@@ -1003,16 +994,16 @@
         <v>5.43</v>
       </c>
       <c r="F13" s="2">
-        <v>1317.7</v>
+        <v>1396.4</v>
       </c>
       <c r="G13" s="2">
-        <v>51.2</v>
+        <v>54.3</v>
       </c>
       <c r="H13" s="3">
-        <v>2.57</v>
+        <v>2.72</v>
       </c>
       <c r="I13" s="4">
-        <v>79.0</v>
+        <v>77.0</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>50</v>
@@ -1029,25 +1020,25 @@
         <v>53</v>
       </c>
       <c r="C14" s="3">
-        <v>27.74</v>
+        <v>27.2</v>
       </c>
       <c r="D14" s="3">
         <v>33.19</v>
       </c>
       <c r="E14" s="3">
-        <v>14.07</v>
+        <v>14.3</v>
       </c>
       <c r="F14" s="2">
-        <v>671.7</v>
+        <v>654.0</v>
       </c>
       <c r="G14" s="2">
-        <v>28.6</v>
+        <v>27.8</v>
       </c>
       <c r="H14" s="3">
-        <v>1.16</v>
+        <v>1.13</v>
       </c>
       <c r="I14" s="4">
-        <v>42.0</v>
+        <v>41.0</v>
       </c>
       <c r="K14" s="2" t="s">
         <v>54</v>
@@ -1061,7 +1052,7 @@
         <v>56</v>
       </c>
       <c r="C15" s="3">
-        <v>10.05</v>
+        <v>9.51</v>
       </c>
       <c r="D15" s="3">
         <v>20.5</v>
@@ -1070,13 +1061,13 @@
         <v>7.15</v>
       </c>
       <c r="F15" s="2">
-        <v>107.8</v>
+        <v>109.1</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>30</v>
       </c>
       <c r="H15" s="3">
-        <v>0.76</v>
+        <v>0.77</v>
       </c>
       <c r="I15" s="4">
         <v>17.0</v>
@@ -1096,22 +1087,22 @@
         <v>60</v>
       </c>
       <c r="C16" s="3">
-        <v>18.91</v>
+        <v>19.28</v>
       </c>
       <c r="D16" s="3">
-        <v>19.35</v>
+        <v>19.36</v>
       </c>
       <c r="E16" s="3">
         <v>7.06</v>
       </c>
       <c r="F16" s="2">
-        <v>601.7</v>
+        <v>600.7</v>
       </c>
       <c r="G16" s="2">
-        <v>35.7</v>
+        <v>35.6</v>
       </c>
       <c r="H16" s="3">
-        <v>2.54</v>
+        <v>2.53</v>
       </c>
       <c r="I16" s="4">
         <v>95.0</v>
@@ -1131,7 +1122,7 @@
         <v>64</v>
       </c>
       <c r="C17" s="3">
-        <v>50.36</v>
+        <v>48.05</v>
       </c>
       <c r="D17" s="3">
         <v>59.42</v>
@@ -1140,13 +1131,13 @@
         <v>32.16</v>
       </c>
       <c r="F17" s="2">
-        <v>379.4</v>
+        <v>363.0</v>
       </c>
       <c r="G17" s="2">
-        <v>21.4</v>
+        <v>20.5</v>
       </c>
       <c r="H17" s="3">
-        <v>0.87</v>
+        <v>0.83</v>
       </c>
       <c r="I17" s="4">
         <v>66.0</v>
@@ -1163,25 +1154,25 @@
         <v>67</v>
       </c>
       <c r="C18" s="3">
-        <v>39.67</v>
+        <v>41.29</v>
       </c>
       <c r="D18" s="3">
-        <v>40.73</v>
+        <v>41.51</v>
       </c>
       <c r="E18" s="3">
-        <v>17.63</v>
+        <v>17.89</v>
       </c>
       <c r="F18" s="2">
-        <v>499.4</v>
+        <v>512.6</v>
       </c>
       <c r="G18" s="2">
-        <v>25.3</v>
+        <v>25.9</v>
       </c>
       <c r="H18" s="3">
-        <v>1.82</v>
+        <v>1.86</v>
       </c>
       <c r="I18" s="4">
-        <v>86.0</v>
+        <v>88.0</v>
       </c>
       <c r="K18" s="2" t="s">
         <v>68</v>
@@ -1195,7 +1186,7 @@
         <v>70</v>
       </c>
       <c r="C19" s="3">
-        <v>78.77</v>
+        <v>49.76</v>
       </c>
       <c r="D19" s="3">
         <v>87.36</v>
@@ -1204,16 +1195,16 @@
         <v>28.64</v>
       </c>
       <c r="F19" s="2">
-        <v>201.4</v>
+        <v>139.8</v>
       </c>
       <c r="G19" s="2">
-        <v>9.1</v>
+        <v>6.3</v>
       </c>
       <c r="H19" s="3">
-        <v>1.59</v>
+        <v>1.1</v>
       </c>
       <c r="I19" s="4">
-        <v>95.0</v>
+        <v>82.0</v>
       </c>
       <c r="K19" s="2" t="s">
         <v>71</v>
@@ -1227,22 +1218,22 @@
         <v>73</v>
       </c>
       <c r="C20" s="3">
-        <v>11.08</v>
+        <v>11.23</v>
       </c>
       <c r="D20" s="3">
         <v>14.5</v>
       </c>
       <c r="E20" s="3">
-        <v>3.44</v>
+        <v>3.61</v>
       </c>
       <c r="F20" s="2">
-        <v>667.0</v>
+        <v>691.1</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>30</v>
       </c>
       <c r="H20" s="3">
-        <v>1.15</v>
+        <v>1.19</v>
       </c>
       <c r="I20" s="4">
         <v>94.0</v>
@@ -1262,25 +1253,25 @@
         <v>76</v>
       </c>
       <c r="C21" s="3">
-        <v>7.17</v>
+        <v>7.74</v>
       </c>
       <c r="D21" s="3">
         <v>9.39</v>
       </c>
       <c r="E21" s="3">
-        <v>3.94</v>
+        <v>3.95</v>
       </c>
       <c r="F21" s="2">
-        <v>468.3</v>
+        <v>500.3</v>
       </c>
       <c r="G21" s="2">
-        <v>23.9</v>
+        <v>25.5</v>
       </c>
       <c r="H21" s="3">
-        <v>1.08</v>
+        <v>1.16</v>
       </c>
       <c r="I21" s="4">
-        <v>88.0</v>
+        <v>91.0</v>
       </c>
       <c r="K21" s="2" t="s">
         <v>77</v>
@@ -1294,25 +1285,25 @@
         <v>79</v>
       </c>
       <c r="C22" s="3">
-        <v>28.48</v>
+        <v>28.55</v>
       </c>
       <c r="D22" s="3">
-        <v>29.5</v>
+        <v>30.45</v>
       </c>
       <c r="E22" s="3">
         <v>15.52</v>
       </c>
       <c r="F22" s="2">
-        <v>391.6</v>
+        <v>398.1</v>
       </c>
       <c r="G22" s="2">
-        <v>16.1</v>
+        <v>16.4</v>
       </c>
       <c r="H22" s="3">
-        <v>1.03</v>
+        <v>1.05</v>
       </c>
       <c r="I22" s="4">
-        <v>84.0</v>
+        <v>85.0</v>
       </c>
       <c r="K22" s="2" t="s">
         <v>80</v>
@@ -1326,7 +1317,7 @@
         <v>82</v>
       </c>
       <c r="C23" s="3">
-        <v>27.5</v>
+        <v>27.0</v>
       </c>
       <c r="D23" s="3">
         <v>31.5</v>
@@ -1344,7 +1335,7 @@
         <v>0.36</v>
       </c>
       <c r="I23" s="4">
-        <v>39.0</v>
+        <v>40.0</v>
       </c>
       <c r="J23" s="2" t="s">
         <v>13</v>
@@ -1361,25 +1352,25 @@
         <v>85</v>
       </c>
       <c r="C24" s="3">
-        <v>42.76</v>
+        <v>37.4</v>
       </c>
       <c r="D24" s="3">
         <v>48.7</v>
       </c>
       <c r="E24" s="3">
-        <v>13.05</v>
+        <v>17.14</v>
       </c>
       <c r="F24" s="2">
-        <v>322.3</v>
+        <v>276.5</v>
       </c>
       <c r="G24" s="2">
-        <v>14.4</v>
+        <v>12.4</v>
       </c>
       <c r="H24" s="3">
-        <v>1.27</v>
+        <v>1.09</v>
       </c>
       <c r="I24" s="4">
-        <v>88.0</v>
+        <v>74.0</v>
       </c>
       <c r="K24" s="2" t="s">
         <v>86</v>
@@ -1393,7 +1384,7 @@
         <v>88</v>
       </c>
       <c r="C25" s="3">
-        <v>11.77</v>
+        <v>11.01</v>
       </c>
       <c r="D25" s="3">
         <v>14.27</v>
@@ -1402,13 +1393,13 @@
         <v>10.68</v>
       </c>
       <c r="F25" s="2">
-        <v>74.9</v>
+        <v>71.8</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>30</v>
       </c>
       <c r="H25" s="3">
-        <v>0.49</v>
+        <v>0.47</v>
       </c>
       <c r="I25" s="4">
         <v>42.0</v>
@@ -1425,7 +1416,7 @@
         <v>91</v>
       </c>
       <c r="C26" s="3">
-        <v>14.13</v>
+        <v>13.95</v>
       </c>
       <c r="D26" s="3">
         <v>23.5</v>
@@ -1434,7 +1425,7 @@
         <v>11.13</v>
       </c>
       <c r="F26" s="2">
-        <v>127.9</v>
+        <v>118.5</v>
       </c>
       <c r="G26" s="2">
         <v>11.9</v>
@@ -1443,7 +1434,7 @@
         <v>1.47</v>
       </c>
       <c r="I26" s="4">
-        <v>32.0</v>
+        <v>29.0</v>
       </c>
       <c r="K26" s="2" t="s">
         <v>92</v>
@@ -1457,94 +1448,60 @@
         <v>94</v>
       </c>
       <c r="C27" s="3">
-        <v>9.37</v>
+        <v>22.0</v>
       </c>
       <c r="D27" s="3">
-        <v>10.52</v>
+        <v>26.77</v>
       </c>
       <c r="E27" s="3">
-        <v>5.22</v>
+        <v>17.61</v>
       </c>
       <c r="F27" s="2">
-        <v>346.5</v>
+        <v>132.0</v>
       </c>
       <c r="G27" s="2">
-        <v>4.9</v>
+        <v>22.3</v>
       </c>
       <c r="H27" s="3">
-        <v>0.55</v>
+        <v>1.06</v>
       </c>
       <c r="I27" s="4">
-        <v>86.0</v>
-      </c>
-      <c r="J27" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="K27" s="2" t="s">
-        <v>95</v>
+        <v>53.0</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="C28" s="3">
+        <v>60.22</v>
+      </c>
+      <c r="D28" s="3">
+        <v>61.94</v>
+      </c>
+      <c r="E28" s="3">
+        <v>22.66</v>
+      </c>
+      <c r="F28" s="2">
+        <v>803.4</v>
+      </c>
+      <c r="G28" s="2">
+        <v>151.4</v>
+      </c>
+      <c r="H28" s="3">
+        <v>2.39</v>
+      </c>
+      <c r="I28" s="4">
+        <v>92.0</v>
+      </c>
+      <c r="K28" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C28" s="3">
-        <v>22.03</v>
-      </c>
-      <c r="D28" s="3">
-        <v>26.77</v>
-      </c>
-      <c r="E28" s="3">
-        <v>17.61</v>
-      </c>
-      <c r="F28" s="2">
-        <v>133.0</v>
-      </c>
-      <c r="G28" s="2">
-        <v>22.5</v>
-      </c>
-      <c r="H28" s="3">
-        <v>1.07</v>
-      </c>
-      <c r="I28" s="4">
-        <v>52.0</v>
-      </c>
-    </row>
-    <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="B29" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="C29" s="3">
-        <v>60.62</v>
-      </c>
-      <c r="D29" s="3">
-        <v>61.46</v>
-      </c>
-      <c r="E29" s="3">
-        <v>21.29</v>
-      </c>
-      <c r="F29" s="2">
-        <v>806.1</v>
-      </c>
-      <c r="G29" s="2">
-        <v>151.9</v>
-      </c>
-      <c r="H29" s="3">
-        <v>2.39</v>
-      </c>
-      <c r="I29" s="4">
-        <v>93.0</v>
-      </c>
-      <c r="K29" s="2" t="s">
-        <v>100</v>
-      </c>
-    </row>
+    </row>
+    <row r="29" ht="15.75" customHeight="1"/>
     <row r="30" ht="15.75" customHeight="1"/>
     <row r="31" ht="15.75" customHeight="1"/>
     <row r="32" ht="15.75" customHeight="1"/>

</xml_diff>